<commit_message>
update question 10, 11, 12, 13, 14
</commit_message>
<xml_diff>
--- a/Homework2/my-simulation/question7.xlsx
+++ b/Homework2/my-simulation/question7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Document_forme\project_tiny\Cource_report\DTUD\Homework2\my-simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD4C922-0925-4C67-AF61-8B75B198DD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBBF57B-AFB5-458B-BF4A-BD9348BC8BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B2724B8F-81E9-4CBD-8F1B-A41AC1296333}"/>
   </bookViews>
@@ -92,8 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -467,14 +466,14 @@
         <f>B2-C2</f>
         <v>2.8057829740135709E-8</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="1">
-        <f>MIN($D:$D)</f>
-        <v>-2.9118879475431569E-6</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="H2">
+        <f>MAX($D:$D)</f>
+        <v>2.8057829740135709E-8</v>
+      </c>
+      <c r="I2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -493,14 +492,14 @@
         <f t="shared" ref="D3:D66" si="1">B3-C3</f>
         <v>-5.2560556323966168E-9</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="1">
-        <f>MAX($D:$D)</f>
-        <v>2.8057829740135709E-8</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="H3">
+        <f>MIN($D:$D)</f>
+        <v>-2.9118879475431569E-6</v>
+      </c>
+      <c r="I3" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>